<commit_message>
update ER dashboard data 2026-07-01 12:44
</commit_message>
<xml_diff>
--- a/docs/reports/daily/ER_Kavach_Unified_KPI_Jun29-Jun29.xlsx
+++ b/docs/reports/daily/ER_Kavach_Unified_KPI_Jun29-Jun29.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified KPI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EB Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Degradation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KM Verification" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Unified KPI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EB Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mode Degradation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="KM Verification" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3970,7 +3970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:M110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4048,6 +4048,11 @@
           <t>Valid Trip?</t>
         </is>
       </c>
+      <c r="M5" s="14" t="inlineStr">
+        <is>
+          <t>Loco Travel</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="31" t="inlineStr">
@@ -4104,6 +4109,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M6" s="16" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="31" t="inlineStr">
@@ -4160,6 +4166,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M7" s="16" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
@@ -4216,6 +4223,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M8" s="16" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="31" t="inlineStr">
@@ -4272,6 +4280,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M9" s="16" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="31" t="inlineStr">
@@ -4328,6 +4337,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M10" s="16" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="31" t="inlineStr">
@@ -4384,6 +4394,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M11" s="16" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="31" t="inlineStr">
@@ -4440,6 +4451,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M12" s="16" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
@@ -4496,6 +4508,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M13" s="16" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="31" t="inlineStr">
@@ -4552,6 +4565,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M14" s="16" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="31" t="inlineStr">
@@ -4608,6 +4622,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M15" s="16" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="31" t="inlineStr">
@@ -4664,6 +4679,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M16" s="16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
@@ -4720,6 +4736,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M17" s="16" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="31" t="inlineStr">
@@ -4776,6 +4793,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M18" s="16" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="31" t="inlineStr">
@@ -4832,6 +4850,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M19" s="16" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
@@ -4888,6 +4907,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M20" s="16" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
@@ -4944,6 +4964,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M21" s="16" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="31" t="inlineStr">
@@ -5000,6 +5021,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M22" s="16" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="31" t="inlineStr">
@@ -5056,6 +5078,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M23" s="16" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="31" t="inlineStr">
@@ -5112,6 +5135,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M24" s="16" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="31" t="inlineStr">
@@ -5168,6 +5192,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M25" s="16" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
@@ -5224,6 +5249,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M26" s="16" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
@@ -5280,6 +5306,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M27" s="16" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="31" t="inlineStr">
@@ -5336,6 +5363,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M28" s="16" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
@@ -5392,6 +5420,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M29" s="16" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="31" t="inlineStr">
@@ -5448,6 +5477,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M30" s="16" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -5504,6 +5534,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M31" s="16" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="31" t="inlineStr">
@@ -5560,6 +5591,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M32" s="16" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="31" t="inlineStr">
@@ -5616,6 +5648,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M33" s="16" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="31" t="inlineStr">
@@ -5672,6 +5705,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M34" s="16" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="31" t="inlineStr">
@@ -5728,6 +5762,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M35" s="16" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -5784,6 +5819,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M36" s="16" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -5840,6 +5876,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M37" s="16" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -5896,6 +5933,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M38" s="16" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
@@ -5952,6 +5990,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M39" s="16" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="31" t="inlineStr">
@@ -6008,6 +6047,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M40" s="16" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="31" t="inlineStr">
@@ -6064,6 +6104,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M41" s="16" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="31" t="inlineStr">
@@ -6120,6 +6161,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M42" s="16" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
@@ -6176,6 +6218,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M43" s="16" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="31" t="inlineStr">
@@ -6232,6 +6275,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M44" s="16" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
@@ -6288,6 +6332,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M45" s="16" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -6344,6 +6389,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M46" s="16" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
@@ -6400,6 +6446,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M47" s="16" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
@@ -6456,6 +6503,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
@@ -6512,6 +6560,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="31" t="inlineStr">
@@ -6568,6 +6617,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M50" s="16" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="31" t="inlineStr">
@@ -6624,6 +6674,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M51" s="16" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="31" t="inlineStr">
@@ -6680,6 +6731,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M52" s="16" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="31" t="inlineStr">
@@ -6736,6 +6788,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M53" s="16" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
@@ -6792,6 +6845,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M54" s="16" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="31" t="inlineStr">
@@ -6848,6 +6902,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M55" s="16" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="31" t="inlineStr">
@@ -6904,6 +6959,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M56" s="16" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
@@ -6960,6 +7016,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M57" s="16" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
@@ -7016,6 +7073,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M58" s="16" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="31" t="inlineStr">
@@ -7072,6 +7130,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M59" s="16" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
@@ -7128,6 +7187,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M60" s="16" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
@@ -7184,6 +7244,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M61" s="16" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
@@ -7240,6 +7301,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M62" s="16" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="31" t="inlineStr">
@@ -7296,6 +7358,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M63" s="16" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="31" t="inlineStr">
@@ -7352,6 +7415,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M64" s="16" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="31" t="inlineStr">
@@ -7408,6 +7472,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M65" s="16" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="31" t="inlineStr">
@@ -7464,6 +7529,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M66" s="16" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="31" t="inlineStr">
@@ -7520,6 +7586,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M67" s="16" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
@@ -7576,6 +7643,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M68" s="16" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -7632,6 +7700,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M69" s="16" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
@@ -7688,6 +7757,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M70" s="16" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
@@ -7744,6 +7814,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M71" s="16" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
@@ -7800,6 +7871,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M72" s="16" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
@@ -7856,6 +7928,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M73" s="16" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="31" t="inlineStr">
@@ -7912,6 +7985,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M74" s="16" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="31" t="inlineStr">
@@ -7968,6 +8042,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M75" s="16" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="16" t="inlineStr">
@@ -8024,6 +8099,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M76" s="16" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="31" t="inlineStr">
@@ -8080,6 +8156,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M77" s="16" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
@@ -8136,6 +8213,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M78" s="16" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
@@ -8192,6 +8270,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M79" s="16" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
@@ -8248,6 +8327,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M80" s="16" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="16" t="inlineStr">
@@ -8304,6 +8384,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M81" s="16" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
@@ -8360,6 +8441,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M82" s="16" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
@@ -8416,6 +8498,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M83" s="16" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
@@ -8472,6 +8555,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M84" s="16" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
@@ -8528,6 +8612,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M85" s="16" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
@@ -8584,6 +8669,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M86" s="16" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
@@ -8640,6 +8726,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M87" s="16" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="16" t="inlineStr">
@@ -8696,6 +8783,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M88" s="16" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
@@ -8752,6 +8840,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M89" s="16" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
@@ -8808,6 +8897,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M90" s="16" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
@@ -8864,6 +8954,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M91" s="16" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="31" t="inlineStr">
@@ -8920,6 +9011,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M92" s="16" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="16" t="inlineStr">
@@ -8976,6 +9068,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M93" s="16" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="16" t="inlineStr">
@@ -9032,6 +9125,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M94" s="16" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
@@ -9088,6 +9182,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M95" s="16" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="31" t="inlineStr">
@@ -9144,6 +9239,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M96" s="16" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="31" t="inlineStr">
@@ -9200,6 +9296,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M97" s="16" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="31" t="inlineStr">
@@ -9256,6 +9353,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M98" s="16" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
@@ -9312,6 +9410,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M99" s="16" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
@@ -9368,6 +9467,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M100" s="16" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
@@ -9424,6 +9524,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M101" s="16" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
@@ -9480,6 +9581,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M102" s="16" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
@@ -9536,6 +9638,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M103" s="16" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
@@ -9592,6 +9695,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M104" s="16" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
@@ -9648,6 +9752,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M105" s="16" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
@@ -9704,6 +9809,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M106" s="16" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
@@ -9760,6 +9866,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M107" s="16" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="31" t="inlineStr">
@@ -9816,6 +9923,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M108" s="16" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="31" t="inlineStr">
@@ -9872,6 +9980,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M109" s="16" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="31" t="inlineStr">
@@ -9928,6 +10037,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M110" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
update ER dashboard data 2026-07-01 12:59
</commit_message>
<xml_diff>
--- a/docs/reports/daily/ER_Kavach_Unified_KPI_Jun29-Jun29.xlsx
+++ b/docs/reports/daily/ER_Kavach_Unified_KPI_Jun29-Jun29.xlsx
@@ -4109,7 +4109,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M6" s="16" t="inlineStr"/>
+      <c r="M6" s="16" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="31" t="inlineStr">
@@ -4166,7 +4170,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M7" s="16" t="inlineStr"/>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
@@ -4223,7 +4231,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M8" s="16" t="inlineStr"/>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="31" t="inlineStr">
@@ -4280,7 +4292,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M9" s="16" t="inlineStr"/>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="31" t="inlineStr">
@@ -4337,7 +4353,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M10" s="16" t="inlineStr"/>
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>Howrah</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="31" t="inlineStr">
@@ -4394,7 +4414,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M11" s="16" t="inlineStr"/>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="31" t="inlineStr">
@@ -4451,7 +4475,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M12" s="16" t="inlineStr"/>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
@@ -4508,7 +4536,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M13" s="16" t="inlineStr"/>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="31" t="inlineStr">
@@ -4565,7 +4597,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M14" s="16" t="inlineStr"/>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="31" t="inlineStr">
@@ -4622,7 +4658,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M15" s="16" t="inlineStr"/>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="31" t="inlineStr">
@@ -4679,7 +4719,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M16" s="16" t="inlineStr"/>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
@@ -4736,7 +4780,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M17" s="16" t="inlineStr"/>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="31" t="inlineStr">
@@ -4793,7 +4841,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M18" s="16" t="inlineStr"/>
+      <c r="M18" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="31" t="inlineStr">
@@ -4850,7 +4902,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M19" s="16" t="inlineStr"/>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
@@ -4907,7 +4963,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M20" s="16" t="inlineStr"/>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
@@ -4964,7 +5024,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M21" s="16" t="inlineStr"/>
+      <c r="M21" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="31" t="inlineStr">
@@ -5021,7 +5085,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M22" s="16" t="inlineStr"/>
+      <c r="M22" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="31" t="inlineStr">
@@ -5078,7 +5146,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M23" s="16" t="inlineStr"/>
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="31" t="inlineStr">
@@ -5135,7 +5207,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M24" s="16" t="inlineStr"/>
+      <c r="M24" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="31" t="inlineStr">
@@ -5192,7 +5268,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M25" s="16" t="inlineStr"/>
+      <c r="M25" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
@@ -5249,7 +5329,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M26" s="16" t="inlineStr"/>
+      <c r="M26" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
@@ -5306,7 +5390,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M27" s="16" t="inlineStr"/>
+      <c r="M27" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="31" t="inlineStr">
@@ -5363,7 +5451,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M28" s="16" t="inlineStr"/>
+      <c r="M28" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
@@ -5420,7 +5512,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M29" s="16" t="inlineStr"/>
+      <c r="M29" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="31" t="inlineStr">
@@ -5477,7 +5573,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M30" s="16" t="inlineStr"/>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -5534,7 +5634,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M31" s="16" t="inlineStr"/>
+      <c r="M31" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="31" t="inlineStr">
@@ -5591,7 +5695,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M32" s="16" t="inlineStr"/>
+      <c r="M32" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="31" t="inlineStr">
@@ -5648,7 +5756,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M33" s="16" t="inlineStr"/>
+      <c r="M33" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="31" t="inlineStr">
@@ -5705,7 +5817,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M34" s="16" t="inlineStr"/>
+      <c r="M34" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="31" t="inlineStr">
@@ -5762,7 +5878,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M35" s="16" t="inlineStr"/>
+      <c r="M35" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -5819,7 +5939,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M36" s="16" t="inlineStr"/>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -5876,7 +6000,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M37" s="16" t="inlineStr"/>
+      <c r="M37" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -5933,7 +6061,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M38" s="16" t="inlineStr"/>
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
@@ -5990,7 +6122,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M39" s="16" t="inlineStr"/>
+      <c r="M39" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="31" t="inlineStr">
@@ -6047,7 +6183,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M40" s="16" t="inlineStr"/>
+      <c r="M40" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="31" t="inlineStr">
@@ -6104,7 +6244,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M41" s="16" t="inlineStr"/>
+      <c r="M41" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="31" t="inlineStr">
@@ -6161,7 +6305,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M42" s="16" t="inlineStr"/>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
@@ -6218,7 +6366,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M43" s="16" t="inlineStr"/>
+      <c r="M43" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="31" t="inlineStr">
@@ -6275,7 +6427,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M44" s="16" t="inlineStr"/>
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
@@ -6332,7 +6488,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M45" s="16" t="inlineStr"/>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -6389,7 +6549,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M46" s="16" t="inlineStr"/>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
@@ -6446,7 +6610,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M47" s="16" t="inlineStr"/>
+      <c r="M47" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
@@ -6503,7 +6671,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M48" s="16" t="inlineStr"/>
+      <c r="M48" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
@@ -6560,7 +6732,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M49" s="16" t="inlineStr"/>
+      <c r="M49" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="31" t="inlineStr">
@@ -6617,7 +6793,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M50" s="16" t="inlineStr"/>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="31" t="inlineStr">
@@ -6674,7 +6854,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M51" s="16" t="inlineStr"/>
+      <c r="M51" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="31" t="inlineStr">
@@ -6731,7 +6915,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M52" s="16" t="inlineStr"/>
+      <c r="M52" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="31" t="inlineStr">
@@ -6788,7 +6976,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M53" s="16" t="inlineStr"/>
+      <c r="M53" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
@@ -6845,7 +7037,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M54" s="16" t="inlineStr"/>
+      <c r="M54" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="31" t="inlineStr">
@@ -6902,7 +7098,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M55" s="16" t="inlineStr"/>
+      <c r="M55" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="31" t="inlineStr">
@@ -6959,7 +7159,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M56" s="16" t="inlineStr"/>
+      <c r="M56" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
@@ -7016,7 +7220,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M57" s="16" t="inlineStr"/>
+      <c r="M57" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
@@ -7073,7 +7281,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M58" s="16" t="inlineStr"/>
+      <c r="M58" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="31" t="inlineStr">
@@ -7130,7 +7342,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M59" s="16" t="inlineStr"/>
+      <c r="M59" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
@@ -7187,7 +7403,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M60" s="16" t="inlineStr"/>
+      <c r="M60" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
@@ -7244,7 +7464,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M61" s="16" t="inlineStr"/>
+      <c r="M61" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
@@ -7301,7 +7525,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M62" s="16" t="inlineStr"/>
+      <c r="M62" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="31" t="inlineStr">
@@ -7358,7 +7586,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M63" s="16" t="inlineStr"/>
+      <c r="M63" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="31" t="inlineStr">
@@ -7415,7 +7647,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M64" s="16" t="inlineStr"/>
+      <c r="M64" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="31" t="inlineStr">
@@ -7472,7 +7708,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M65" s="16" t="inlineStr"/>
+      <c r="M65" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="31" t="inlineStr">
@@ -7529,7 +7769,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M66" s="16" t="inlineStr"/>
+      <c r="M66" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="31" t="inlineStr">
@@ -7586,7 +7830,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M67" s="16" t="inlineStr"/>
+      <c r="M67" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
@@ -7643,7 +7891,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M68" s="16" t="inlineStr"/>
+      <c r="M68" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -7700,7 +7952,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M69" s="16" t="inlineStr"/>
+      <c r="M69" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="31" t="inlineStr">
@@ -7757,7 +8013,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M70" s="16" t="inlineStr"/>
+      <c r="M70" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
@@ -7814,7 +8074,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M71" s="16" t="inlineStr"/>
+      <c r="M71" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
@@ -7871,7 +8135,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M72" s="16" t="inlineStr"/>
+      <c r="M72" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
@@ -7928,7 +8196,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M73" s="16" t="inlineStr"/>
+      <c r="M73" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="31" t="inlineStr">
@@ -7985,7 +8257,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M74" s="16" t="inlineStr"/>
+      <c r="M74" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="31" t="inlineStr">
@@ -8042,7 +8318,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M75" s="16" t="inlineStr"/>
+      <c r="M75" s="16" t="inlineStr">
+        <is>
+          <t>Barddhaman Jn, Talit</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="16" t="inlineStr">
@@ -8099,7 +8379,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M76" s="16" t="inlineStr"/>
+      <c r="M76" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="31" t="inlineStr">
@@ -8156,7 +8440,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M77" s="16" t="inlineStr"/>
+      <c r="M77" s="16" t="inlineStr">
+        <is>
+          <t>Barddhaman Jn, Talit</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="31" t="inlineStr">
@@ -8213,7 +8501,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M78" s="16" t="inlineStr"/>
+      <c r="M78" s="16" t="inlineStr">
+        <is>
+          <t>Barddhaman Jn, Talit</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
@@ -8270,7 +8562,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M79" s="16" t="inlineStr"/>
+      <c r="M79" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
@@ -8327,7 +8623,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M80" s="16" t="inlineStr"/>
+      <c r="M80" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="16" t="inlineStr">
@@ -8384,7 +8684,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M81" s="16" t="inlineStr"/>
+      <c r="M81" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
@@ -8441,7 +8745,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M82" s="16" t="inlineStr"/>
+      <c r="M82" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="31" t="inlineStr">
@@ -8498,7 +8806,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M83" s="16" t="inlineStr"/>
+      <c r="M83" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
@@ -8555,7 +8867,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M84" s="16" t="inlineStr"/>
+      <c r="M84" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
@@ -8612,7 +8928,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M85" s="16" t="inlineStr"/>
+      <c r="M85" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
@@ -8669,7 +8989,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M86" s="16" t="inlineStr"/>
+      <c r="M86" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
@@ -8726,7 +9050,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M87" s="16" t="inlineStr"/>
+      <c r="M87" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="16" t="inlineStr">
@@ -8783,7 +9111,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M88" s="16" t="inlineStr"/>
+      <c r="M88" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
@@ -8840,7 +9172,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M89" s="16" t="inlineStr"/>
+      <c r="M89" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="31" t="inlineStr">
@@ -8897,7 +9233,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M90" s="16" t="inlineStr"/>
+      <c r="M90" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="31" t="inlineStr">
@@ -8954,7 +9294,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M91" s="16" t="inlineStr"/>
+      <c r="M91" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="31" t="inlineStr">
@@ -9011,7 +9355,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M92" s="16" t="inlineStr"/>
+      <c r="M92" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="16" t="inlineStr">
@@ -9068,7 +9416,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M93" s="16" t="inlineStr"/>
+      <c r="M93" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="16" t="inlineStr">
@@ -9125,7 +9477,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M94" s="16" t="inlineStr"/>
+      <c r="M94" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
@@ -9182,7 +9538,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M95" s="16" t="inlineStr"/>
+      <c r="M95" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="31" t="inlineStr">
@@ -9239,7 +9599,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M96" s="16" t="inlineStr"/>
+      <c r="M96" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="31" t="inlineStr">
@@ -9296,7 +9660,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M97" s="16" t="inlineStr"/>
+      <c r="M97" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="31" t="inlineStr">
@@ -9353,7 +9721,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M98" s="16" t="inlineStr"/>
+      <c r="M98" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="31" t="inlineStr">
@@ -9410,7 +9782,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M99" s="16" t="inlineStr"/>
+      <c r="M99" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="31" t="inlineStr">
@@ -9467,7 +9843,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M100" s="16" t="inlineStr"/>
+      <c r="M100" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
@@ -9524,7 +9904,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M101" s="16" t="inlineStr"/>
+      <c r="M101" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
@@ -9581,7 +9965,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M102" s="16" t="inlineStr"/>
+      <c r="M102" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
@@ -9638,7 +10026,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M103" s="16" t="inlineStr"/>
+      <c r="M103" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
@@ -9695,7 +10087,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M104" s="16" t="inlineStr"/>
+      <c r="M104" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="31" t="inlineStr">
@@ -9752,7 +10148,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M105" s="16" t="inlineStr"/>
+      <c r="M105" s="16" t="inlineStr">
+        <is>
+          <t>Howrah, Howrah Sorting Yard, Liluah, Belur, Bally, Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="31" t="inlineStr">
@@ -9809,7 +10209,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M106" s="16" t="inlineStr"/>
+      <c r="M106" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="31" t="inlineStr">
@@ -9866,7 +10270,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M107" s="16" t="inlineStr"/>
+      <c r="M107" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn, Talit, LC-59, Khana Jn, Khana Link, Galsi, LC-83, Paraj, Mankar, LC-96, Panagarh, LC-105, Rajbandh, LC-111, Durgapur, DCOP, Waria, Andal East Outer, Andal, Baktarnagar B H, Raniganj, Nimcha B H, Ratibati, Kaliphari, Asansol, Barachak Jn, Sitarampur Central, Kulti, Barakar, Kumardubi, Mugma, Thaparnagar, Kalubathan, LC-12, Chhota Ambana</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="31" t="inlineStr">
@@ -9923,7 +10331,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M108" s="16" t="inlineStr"/>
+      <c r="M108" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="31" t="inlineStr">
@@ -9980,7 +10392,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M109" s="16" t="inlineStr"/>
+      <c r="M109" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni, LC-12, Janai Road, Baruipara, Kamarkundu, LC-31, Chandanpur, LC-38, Belmuri, Cheragram, LC-41, Gurap, LC-48, Jaugram, LC-57, Masagram, Palla Road, Saktigarh, Gangpur, Barddhaman Jn</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="31" t="inlineStr">
@@ -10037,7 +10453,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M110" s="16" t="inlineStr"/>
+      <c r="M110" s="16" t="inlineStr">
+        <is>
+          <t>Belanagar, Dankuni</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>